<commit_message>
Use Q/S × L × (W + G) for floor-pallet area with gangways
</commit_message>
<xml_diff>
--- a/LogEn_Shift_Inventory_Template.xlsx
+++ b/LogEn_Shift_Inventory_Template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Part Number</t>
   </si>
@@ -86,7 +86,10 @@
     <t>Use one unique part number per row. Invalid and duplicate rows remain visible. Both floor and rack scenarios use the same required pallets.</t>
   </si>
   <si>
-    <t>Each part has dedicated floor rows and rack bays. Gangway-inclusive figures use the full (100%) configured gangway width for allocated planning estimates, not optimized physical layouts.</t>
+    <t>Floor with gangways = (Q / S) × L × (W + G) / 1,000,000; Q = required pallets, S = effective floor stacking, L/W/G in mm. Keep Q / S unrounded and use full gangway width G.</t>
+  </si>
+  <si>
+    <t>Floor without gangways retains actual occupied rows and clearances. Rack gangways retain actual rack run frontage × full gangway width. These are allocated planning estimates, not optimized layouts.</t>
   </si>
   <si>
     <t>All imports, calculations, projects and exports work offline on this device.</t>
@@ -556,7 +559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
@@ -647,6 +650,11 @@
         <v>25</v>
       </c>
     </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Round selected-shift daily pallet demand and add per-part Stackability controls
</commit_message>
<xml_diff>
--- a/LogEn_Shift_Inventory_Template.xlsx
+++ b/LogEn_Shift_Inventory_Template.xlsx
@@ -56,10 +56,10 @@
     <t>DOH (Days on hand) = required coverage days for that part. Choose input DOH or a custom project DOH override.</t>
   </si>
   <si>
-    <t>Required pallets = CEILING(CEILING(Consumption per shift / QTY in Box / QTY boxes per Pallet) × selected DOH × shifts per day).</t>
-  </si>
-  <si>
-    <t>The inner CEILING rounds pallets for one shift up first. Do not replace this with one final rounding of fractional daily demand.</t>
+    <t>Required pallets = CEILING(CEILING(Consumption per shift / QTY in Box / QTY boxes per Pallet × shifts per day) × selected DOH).</t>
+  </si>
+  <si>
+    <t>Multiply the raw pallet demand per shift by the selected 1, 2 or 3 shifts first, then round the combined daily pallet demand up once. Apply DOH after that daily rounding.</t>
   </si>
   <si>
     <t>Shifts per day must be 1, 2 or 3; the default is 2. Custom project DOH defaults to 5 days.</t>
@@ -68,7 +68,7 @@
     <t>L(mm), W(mm) and H(mm) are loaded pallet dimensions in millimeters.</t>
   </si>
   <si>
-    <t>The eight-column template omits stacking: floor stacking defaults to 1. An optional extra Stacking column is supported, and stacking can be edited manually.</t>
+    <t>The eight-column template omits stacking: floor stacking defaults to 1. An optional extra Stacking column is supported. Enable Stackability in Shifts &amp; days on hand to edit and apply the saved factor for each part; unchecked uses effective stacking 1 without erasing saved factors.</t>
   </si>
   <si>
     <t>Current stock quantity is optional. If absent, actual stock coverage remains unavailable rather than being treated as zero stock.</t>

</xml_diff>

<commit_message>
Update Excel template guidance for decimal pallet quantities
</commit_message>
<xml_diff>
--- a/LogEn_Shift_Inventory_Template.xlsx
+++ b/LogEn_Shift_Inventory_Template.xlsx
@@ -56,10 +56,10 @@
     <t>DOH (Days on hand) = required coverage days for that part. Choose input DOH or a custom project DOH override.</t>
   </si>
   <si>
-    <t>Required pallets = CEILING(CEILING(Consumption per shift / QTY in Box / QTY boxes per Pallet × shifts per day) × selected DOH).</t>
-  </si>
-  <si>
-    <t>Multiply the raw pallet demand per shift by the selected 1, 2 or 3 shifts first, then round the combined daily pallet demand up once. Apply DOH after that daily rounding.</t>
+    <t>Required pallets = consumption per shift / parts per box / boxes per pallet × shifts per day × DOH. Decimal quantities retained; only physical capacity units round up.</t>
+  </si>
+  <si>
+    <t>Multiply raw pallet demand per shift by selected shifts and DOH without rounding.</t>
   </si>
   <si>
     <t>Shifts per day must be 1, 2 or 3; the default is 2. Custom project DOH defaults to 5 days.</t>
@@ -77,7 +77,7 @@
     <t>Old monthly and daily templates remain supported with explicit conversion notices. Legacy consumption is converted once using the production settings selected at import.</t>
   </si>
   <si>
-    <t>If old data has only direct parts-per-pallet capacity, packaging is inferred as one box containing that capacity. Review inferred packaging before relying on shift rounding.</t>
+    <t>If old data has only direct parts-per-pallet capacity, packaging is inferred as one box containing that capacity. Review inferred packaging before using calculated demand.</t>
   </si>
   <si>
     <t>Use numeric cells or decimal-point text. Formula cells are not evaluated; paste calculated values before importing.</t>
@@ -86,7 +86,7 @@
     <t>Use one unique part number per row. Invalid and duplicate rows remain visible. Both floor and rack scenarios use the same required pallets.</t>
   </si>
   <si>
-    <t>Floor with gangways = (Q / S) × L × (W + G) / 1,000,000; Q = required pallets, S = effective floor stacking, L/W/G in mm. Keep Q / S unrounded and use full gangway width G.</t>
+    <t>GS with gangway = GS net + lane width (mm) * lanes * physical gangway (m) / 2000.</t>
   </si>
   <si>
     <t>Floor without gangways retains actual occupied rows and clearances. Its project total sums each independently valid floor storage result rounded to two decimals; rack fit errors do not remove valid floor areas. Rack gangways retain actual rack run frontage × full gangway width. These are allocated planning estimates, not optimized layouts.</t>

</xml_diff>

<commit_message>
Round required pallets only after multiplying raw demand by shifts and DOH
</commit_message>
<xml_diff>
--- a/LogEn_Shift_Inventory_Template.xlsx
+++ b/LogEn_Shift_Inventory_Template.xlsx
@@ -56,10 +56,10 @@
     <t>DOH (Days on hand) = required coverage days for that part. Choose input DOH or a custom project DOH override.</t>
   </si>
   <si>
-    <t>Required pallets = consumption per shift / parts per box / boxes per pallet × shifts per day × DOH. Decimal quantities retained; only physical capacity units round up.</t>
-  </si>
-  <si>
-    <t>Multiply raw pallet demand per shift by selected shifts and DOH without rounding.</t>
+    <t>Required pallets = consumption per shift / parts per box / boxes per pallet × shifts per day × DOH. Keep all intermediate decimals; round up only the final required pallet quantity.</t>
+  </si>
+  <si>
+    <t>Multiply raw pallet demand per shift by selected shifts and DOH without intermediate rounding; round up only the final required pallets.</t>
   </si>
   <si>
     <t>Shifts per day must be 1, 2 or 3; the default is 2. Custom project DOH defaults to 5 days.</t>

</xml_diff>

<commit_message>
Add per-rack storage policies, deletion and category planning filters
</commit_message>
<xml_diff>
--- a/LogEn_Shift_Inventory_Template.xlsx
+++ b/LogEn_Shift_Inventory_Template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Part Number</t>
   </si>
@@ -38,13 +38,19 @@
     <t>H(mm)</t>
   </si>
   <si>
+    <t>Category</t>
+  </si>
+  <si>
     <t>SAMPLE-001</t>
   </si>
   <si>
+    <t>Bulk</t>
+  </si>
+  <si>
     <t>LogEn — warehouse input template</t>
   </si>
   <si>
-    <t>Keep exactly these eight template headings. Replace or delete SAMPLE-001 before adding your parts.</t>
+    <t>Keep these nine template headings (Category is optional when importing older files). Replace or delete SAMPLE-001 before adding your parts.</t>
   </si>
   <si>
     <t>QTY in Box = individual parts in one box. QTY boxes per Pallet = boxes on one pallet.</t>
@@ -68,7 +74,7 @@
     <t>L(mm), W(mm) and H(mm) are loaded pallet dimensions in millimeters.</t>
   </si>
   <si>
-    <t>The eight-column template omits stacking: floor stacking defaults to 1. An optional extra Stacking column is supported. Choose imported stacking in Part details to use saved factors, automatic height calculation, or one global manual factor.</t>
+    <t>The template omits stacking: floor stacking defaults to 1. An optional extra Stacking column is supported. Choose imported stacking in Part details to use saved factors, automatic height calculation, or one global manual factor.</t>
   </si>
   <si>
     <t>Current stock quantity is optional. If absent, actual stock coverage remains unavailable rather than being treated as zero stock.</t>
@@ -491,14 +497,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="8" width="24" customWidth="1"/>
+    <col min="2" max="9" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="34" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -523,10 +529,13 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2">
         <v>20</v>
@@ -549,9 +558,12 @@
       <c r="H2" s="2">
         <v>1000</v>
       </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -567,92 +579,92 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>